<commit_message>
Entregable 3 y Presentaciones
</commit_message>
<xml_diff>
--- a/docs/Entregable3/Registro_Gestion_Riesgos_SAML.xlsx
+++ b/docs/Entregable3/Registro_Gestion_Riesgos_SAML.xlsx
@@ -1,38 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30606"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDC42092-3976-4073-9AB6-6122A5D24F49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB789FF1-E4D1-40F9-B323-A8FA239B5472}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
     <sheet name="Registro de Riesgos" sheetId="2" r:id="rId2"/>
-    <sheet name="Matriz de Probabilidad-Impacto" sheetId="3" r:id="rId3"/>
-    <sheet name="Guía y Escalas" sheetId="4" r:id="rId4"/>
+    <sheet name="Seguimiento de Riesgo" sheetId="5" r:id="rId3"/>
+    <sheet name="Matriz de Probabilidad-Impacto" sheetId="3" r:id="rId4"/>
+    <sheet name="Guía y Escalas" sheetId="4" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191028" iterateDelta="1E-4"/>
+  <calcPr calcId="179021" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -42,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="180">
   <si>
     <t>Plantilla de Registro y Gestión de Riesgos</t>
   </si>
@@ -143,6 +133,7 @@
         <sz val="10"/>
         <color rgb="FFFFFFFF"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Riesgo (causa → evento → efecto)
 </t>
@@ -152,6 +143,7 @@
         <sz val="10"/>
         <color rgb="FFFFFFFF"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Colores para marcar causa, evento y efecto (no significan positivo o negativo)</t>
     </r>
@@ -210,6 +202,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Integración con API externa</t>
     </r>
@@ -218,6 +211,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">: </t>
     </r>
@@ -226,6 +220,7 @@
         <sz val="9.5"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Debido a la dependencia de una API externa y a la posibilidad de fallos en su disponibilidad</t>
     </r>
@@ -234,6 +229,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>,</t>
     </r>
@@ -242,6 +238,7 @@
         <sz val="9.5"/>
         <color rgb="FFFFC000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> las solicitudes de extracción de datos podrían fallar o exceder el tiempo de espera, </t>
     </r>
@@ -250,6 +247,7 @@
         <sz val="9.5"/>
         <color rgb="FF00B050"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>provocando interrupciones en la ingesta de información y retrasos en la actualización de los datos de oportunidades de contratación.</t>
     </r>
@@ -283,6 +281,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Calidad y normalización de datos</t>
     </r>
@@ -291,6 +290,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">: </t>
     </r>
@@ -299,6 +299,7 @@
         <sz val="9.5"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Debido a la heterogeneidad y posible inconsistencia de los datos recibidos desde la API externa,</t>
     </r>
@@ -307,6 +308,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -315,6 +317,7 @@
         <sz val="9.5"/>
         <color rgb="FFFFC000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>podrían ingresar registros con NIT inválidos, entidades duplicadas, montos incorrectos o códigos UNSPSC/DANE no normalizados</t>
     </r>
@@ -323,6 +326,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -331,6 +335,7 @@
         <sz val="9.5"/>
         <color rgb="FF00B050"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>afectando la confiabilidad de los resultados y la precisión de las oportunidades identificadas.</t>
     </r>
@@ -355,6 +360,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Criterios de filtrado comercial</t>
     </r>
@@ -363,6 +369,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">: </t>
     </r>
@@ -371,6 +378,7 @@
         <sz val="9.5"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Debido a la falta de validación oportuna de los criterios de filtrado con el Product Owner</t>
     </r>
@@ -379,6 +387,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -387,6 +396,7 @@
         <sz val="9.5"/>
         <color rgb="FFFFC000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>podrían aplicarse parámetros incorrectos de UNSPSC, cuantías o zonas geográficas</t>
     </r>
@@ -395,6 +405,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -403,6 +414,7 @@
         <sz val="9.5"/>
         <color rgb="FF00B050"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>ocasionando que se descarten oportunidades relevantes o se presenten resultados poco pertinentes para el equipo comercial.</t>
     </r>
@@ -433,6 +445,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Adopción por parte del equipo comercial:</t>
     </r>
@@ -441,6 +454,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -449,6 +463,7 @@
         <sz val="9.5"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Debido a una capacitación insuficiente o a la falta de apropiación de la herramienta por parte del equipo comercial</t>
     </r>
@@ -457,6 +472,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -465,6 +481,7 @@
         <sz val="9.5"/>
         <color rgb="FFFFC000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>los usuarios podrían no utilizar correctamente los resultados o continuar dependiendo exclusivamente de procesos manuales</t>
     </r>
@@ -473,6 +490,7 @@
         <sz val="9.5"/>
         <color rgb="FF26324A"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -481,6 +499,7 @@
         <sz val="9.5"/>
         <color rgb="FF00B050"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>reduciendo el aprovechamiento de la solución y los beneficios esperados del proyecto.</t>
     </r>
@@ -508,6 +527,7 @@
         <sz val="9.5"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Acceso a la API del CRM</t>
     </r>
@@ -516,6 +536,7 @@
         <sz val="9.5"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">: </t>
     </r>
@@ -524,6 +545,7 @@
         <sz val="9.5"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Debido a la dependencia de la autorización y disponibilidad de acceso a la API del CRM</t>
     </r>
@@ -532,6 +554,7 @@
         <sz val="9.5"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -540,6 +563,7 @@
         <sz val="9.5"/>
         <color rgb="FFFFC000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>podría no ser posible implementar la integración dentro del plazo previsto</t>
     </r>
@@ -548,6 +572,7 @@
         <sz val="9.5"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -556,6 +581,7 @@
         <sz val="9.5"/>
         <color rgb="FF00B050"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>generando retrasos en el alcance del proyecto y obligando a utilizar un mecanismo alternativo de carga de información.</t>
     </r>
@@ -583,6 +609,7 @@
         <sz val="9.5"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Despliegue reproducible con Docker</t>
     </r>
@@ -591,6 +618,7 @@
         <sz val="9.5"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>:</t>
     </r>
@@ -599,6 +627,7 @@
         <sz val="9.5"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> Debido a la ausencia de un entorno de ejecución estandarizado entre n8n y Python</t>
     </r>
@@ -607,6 +636,7 @@
         <sz val="9.5"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -615,6 +645,7 @@
         <sz val="9.5"/>
         <color rgb="FFFFC000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>podrían presentarse diferencias de configuración o dependencias al desplegar la solución en la infraestructura de GRECO</t>
     </r>
@@ -623,6 +654,7 @@
         <sz val="9.5"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -631,6 +663,7 @@
         <sz val="9.5"/>
         <color rgb="FF00B050"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>provocando errores de ejecución, incompatibilidades y mayores tiempos de mantenimiento.</t>
     </r>
@@ -902,13 +935,105 @@
   </si>
   <si>
     <t>Nota — Escalar: cuando un riesgo (amenaza u oportunidad) supera la autoridad del líder de proyecto o el alcance del proyecto, debe escalarse al sponsor, comité o PMO en lugar de gestionarse solo dentro del equipo.</t>
+  </si>
+  <si>
+    <t>Semana</t>
+  </si>
+  <si>
+    <t>Observación</t>
+  </si>
+  <si>
+    <t>21/09/2026 (creación)</t>
+  </si>
+  <si>
+    <t>Implementado y probado</t>
+  </si>
+  <si>
+    <t>Funcionando con normalidad</t>
+  </si>
+  <si>
+    <r>
+      <t>Se construyó la integración (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>extract.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>api_client.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>config.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). Login y consulta confirmados funcionando, pudiendo extraer la informacion que nos son de utilidad </t>
+    </r>
+  </si>
+  <si>
+    <t>Ejecucion manual del script de ingesta para verificar el estado y funcionamiento de la API. Sin incidentes reportados.</t>
+  </si>
+  <si>
+    <t>22/09 – 27/09</t>
+  </si>
+  <si>
+    <t>28/09 – 04/10</t>
+  </si>
+  <si>
+    <t>05/10 – 11/10</t>
+  </si>
+  <si>
+    <t>Seguimiento de Riesgo</t>
+  </si>
+  <si>
+    <t>Integración con API externa: Debido a la dependencia de una API externa y a la posibilidad de fallos en su disponibilidad, las solicitudes de extracción de datos podrían fallar o exceder el tiempo de espera, provocando interrupciones en la ingesta de información y retrasos en la actualización de los datos de oportunidades de contratación.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="38">
+  <fonts count="41">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1100,54 +1225,84 @@
       <sz val="9.5"/>
       <color rgb="FF26324A"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9.5"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9.5"/>
       <color rgb="FFFFC000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9.5"/>
       <color rgb="FF00B050"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9.5"/>
       <color rgb="FF26324A"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9.5"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9.5"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9.5"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="13">
@@ -1224,7 +1379,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1260,11 +1415,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1379,59 +1549,71 @@
     <xf numFmtId="14" fontId="11" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2134,7 +2316,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:F27"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="6" width="30" customWidth="1"/>
@@ -2142,40 +2324,40 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="24.6">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
     </row>
     <row r="3" spans="2:6" ht="15.6">
-      <c r="B3" s="60" t="s">
+      <c r="B3" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
     </row>
     <row r="5" spans="2:6" ht="15" customHeight="1">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
     </row>
     <row r="6" spans="2:6">
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-    </row>
-    <row r="8" spans="2:6" ht="16.899999999999999">
+      <c r="B6" s="52"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+    </row>
+    <row r="8" spans="2:6" ht="16.8">
       <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
@@ -2185,178 +2367,168 @@
       <c r="C9" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="44" t="s">
+      <c r="D9" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
+      <c r="E9" s="53"/>
+      <c r="F9" s="53"/>
     </row>
     <row r="10" spans="2:6" ht="27.75" customHeight="1">
       <c r="B10" s="4"/>
       <c r="C10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="44" t="s">
+      <c r="D10" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
+      <c r="E10" s="53"/>
+      <c r="F10" s="53"/>
     </row>
     <row r="11" spans="2:6" ht="27.75" customHeight="1">
       <c r="B11" s="5"/>
       <c r="C11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="44" t="s">
+      <c r="D11" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
+      <c r="E11" s="53"/>
+      <c r="F11" s="53"/>
     </row>
     <row r="12" spans="2:6" ht="27.75" customHeight="1">
       <c r="B12" s="6"/>
       <c r="C12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="44" t="s">
+      <c r="D12" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
+      <c r="E12" s="53"/>
+      <c r="F12" s="53"/>
     </row>
     <row r="13" spans="2:6" ht="27.75" customHeight="1">
       <c r="B13" s="7"/>
       <c r="C13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="44" t="s">
+      <c r="D13" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-    </row>
-    <row r="15" spans="2:6" ht="16.899999999999999">
+      <c r="E13" s="53"/>
+      <c r="F13" s="53"/>
+    </row>
+    <row r="15" spans="2:6" ht="16.8">
       <c r="B15" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="25.5" customHeight="1">
-      <c r="B16" s="45" t="s">
+      <c r="B16" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="45"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="45"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="54"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="54"/>
     </row>
     <row r="17" spans="2:6" ht="25.5" customHeight="1">
-      <c r="B17" s="45" t="s">
+      <c r="B17" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="45"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="45"/>
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
     </row>
     <row r="18" spans="2:6" ht="25.5" customHeight="1">
-      <c r="B18" s="45" t="s">
+      <c r="B18" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="45"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
     </row>
     <row r="19" spans="2:6" ht="25.5" customHeight="1">
-      <c r="B19" s="45" t="s">
+      <c r="B19" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="45"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="54"/>
+      <c r="E19" s="54"/>
+      <c r="F19" s="54"/>
     </row>
     <row r="20" spans="2:6" ht="25.5" customHeight="1">
-      <c r="B20" s="45" t="s">
+      <c r="B20" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="45"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="45"/>
+      <c r="C20" s="54"/>
+      <c r="D20" s="54"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="54"/>
     </row>
     <row r="21" spans="2:6" ht="25.5" customHeight="1">
-      <c r="B21" s="45" t="s">
+      <c r="B21" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="45"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45"/>
+      <c r="C21" s="54"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="54"/>
     </row>
     <row r="22" spans="2:6" ht="25.5" customHeight="1">
-      <c r="B22" s="45" t="s">
+      <c r="B22" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-    </row>
-    <row r="24" spans="2:6" ht="16.899999999999999">
-      <c r="B24" s="61" t="s">
+      <c r="C22" s="54"/>
+      <c r="D22" s="54"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="54"/>
+    </row>
+    <row r="24" spans="2:6" ht="16.8">
+      <c r="B24" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="C24" s="61"/>
-      <c r="D24" s="61"/>
-      <c r="E24" s="61"/>
-      <c r="F24" s="61"/>
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
     </row>
     <row r="25" spans="2:6" ht="21.75" customHeight="1">
       <c r="B25" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="44" t="s">
+      <c r="C25" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="44"/>
-      <c r="E25" s="44"/>
-      <c r="F25" s="44"/>
+      <c r="D25" s="53"/>
+      <c r="E25" s="53"/>
+      <c r="F25" s="53"/>
     </row>
     <row r="26" spans="2:6" ht="21.75" customHeight="1">
       <c r="B26" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="44" t="s">
+      <c r="C26" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="44"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
+      <c r="D26" s="53"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="53"/>
     </row>
     <row r="27" spans="2:6" ht="21.75" customHeight="1">
       <c r="B27" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="44" t="s">
+      <c r="C27" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="44"/>
-      <c r="E27" s="44"/>
-      <c r="F27" s="44"/>
+      <c r="D27" s="53"/>
+      <c r="E27" s="53"/>
+      <c r="F27" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B5:F6"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B17:F17"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="C25:F25"/>
     <mergeCell ref="C26:F26"/>
@@ -2366,6 +2538,16 @@
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B5:F6"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -2377,8 +2559,8 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O34"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <dimension ref="A1:O33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
@@ -2395,30 +2577,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="21.75" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="63"/>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-      <c r="N1" s="63"/>
-      <c r="O1" s="63"/>
-    </row>
-    <row r="2" spans="1:15" ht="15"/>
-    <row r="3" spans="1:15" s="55" customFormat="1" ht="31.5" customHeight="1">
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+      <c r="O1" s="57"/>
+    </row>
+    <row r="3" spans="1:15" s="46" customFormat="1" ht="31.5" customHeight="1">
       <c r="A3" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="45" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="9" t="s">
@@ -2461,11 +2642,11 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="118.5">
+    <row r="4" spans="1:15" ht="120">
       <c r="A4" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="B4" s="34" t="s">
         <v>46</v>
       </c>
       <c r="C4" s="34" t="s">
@@ -2515,7 +2696,7 @@
       <c r="A5" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="44" t="s">
         <v>54</v>
       </c>
       <c r="C5" s="34" t="s">
@@ -2561,11 +2742,11 @@
         <v>46308</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="96">
+    <row r="6" spans="1:15" ht="97.2">
       <c r="A6" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="47" t="s">
         <v>59</v>
       </c>
       <c r="C6" s="39" t="s">
@@ -2611,11 +2792,11 @@
         <v>46308</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="107.25">
+    <row r="7" spans="1:15" ht="96">
       <c r="A7" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="56" t="s">
+      <c r="B7" s="47" t="s">
         <v>66</v>
       </c>
       <c r="C7" s="39" t="s">
@@ -2661,11 +2842,11 @@
         <v>46308</v>
       </c>
     </row>
-    <row r="8" spans="1:15" s="55" customFormat="1" ht="130.5">
+    <row r="8" spans="1:15" s="46" customFormat="1" ht="120">
       <c r="A8" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="48" t="s">
         <v>72</v>
       </c>
       <c r="C8" s="39" t="s">
@@ -2711,11 +2892,11 @@
         <v>46296</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="118.5">
+    <row r="9" spans="1:15" ht="108">
       <c r="A9" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="49" t="s">
         <v>78</v>
       </c>
       <c r="C9" s="39" t="s">
@@ -3457,7 +3638,6 @@
       <c r="N33" s="15"/>
       <c r="O33" s="15"/>
     </row>
-    <row r="34" spans="1:15" ht="15"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
@@ -3511,12 +3691,100 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FB86DC2-648A-495E-9ED4-3CFB834C9D64}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="19.44140625" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="33.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="67" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+    </row>
+    <row r="2" spans="1:3" ht="91.8" customHeight="1">
+      <c r="A2" s="68" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="69" t="s">
+        <v>168</v>
+      </c>
+      <c r="B3" s="69" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="69" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="72">
+      <c r="A4" s="70" t="s">
+        <v>170</v>
+      </c>
+      <c r="B4" s="70" t="s">
+        <v>171</v>
+      </c>
+      <c r="C4" s="70" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="57.6">
+      <c r="A5" s="70" t="s">
+        <v>175</v>
+      </c>
+      <c r="B5" s="70" t="s">
+        <v>172</v>
+      </c>
+      <c r="C5" s="70" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="57.6">
+      <c r="A6" s="70" t="s">
+        <v>176</v>
+      </c>
+      <c r="B6" s="70" t="s">
+        <v>172</v>
+      </c>
+      <c r="C6" s="70" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="57.6">
+      <c r="A7" s="70" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" s="70" t="s">
+        <v>172</v>
+      </c>
+      <c r="C7" s="70" t="s">
+        <v>174</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:I20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -3526,36 +3794,36 @@
     <col min="10" max="10" width="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" ht="22.9">
-      <c r="B2" s="64" t="s">
+    <row r="2" spans="1:9" ht="22.8">
+      <c r="B2" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="B3" s="65" t="s">
+      <c r="B3" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="65"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
     </row>
     <row r="5" spans="1:9" ht="15" customHeight="1">
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="61" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
+      <c r="D5" s="61"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="61"/>
+      <c r="G5" s="61"/>
     </row>
     <row r="6" spans="1:9">
       <c r="C6" s="16" t="s">
@@ -3573,13 +3841,13 @@
       <c r="G6" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="H6" s="49" t="s">
+      <c r="H6" s="62" t="s">
         <v>90</v>
       </c>
-      <c r="I6" s="49"/>
+      <c r="I6" s="62"/>
     </row>
     <row r="7" spans="1:9" ht="33.75" customHeight="1">
-      <c r="A7" s="47" t="s">
+      <c r="A7" s="58" t="s">
         <v>91</v>
       </c>
       <c r="B7" s="16" t="s">
@@ -3613,7 +3881,7 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="33.75" customHeight="1">
-      <c r="A8" s="47"/>
+      <c r="A8" s="58"/>
       <c r="B8" s="16" t="s">
         <v>95</v>
       </c>
@@ -3645,7 +3913,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="33.75" customHeight="1">
-      <c r="A9" s="47"/>
+      <c r="A9" s="58"/>
       <c r="B9" s="16" t="s">
         <v>97</v>
       </c>
@@ -3677,7 +3945,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="33.75" customHeight="1">
-      <c r="A10" s="47"/>
+      <c r="A10" s="58"/>
       <c r="B10" s="16" t="s">
         <v>99</v>
       </c>
@@ -3703,7 +3971,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="33.75" customHeight="1">
-      <c r="A11" s="47"/>
+      <c r="A11" s="58"/>
       <c r="B11" s="16" t="s">
         <v>100</v>
       </c>
@@ -3728,16 +3996,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="16.899999999999999">
-      <c r="B14" s="61" t="s">
+    <row r="14" spans="1:9" ht="16.8">
+      <c r="B14" s="55" t="s">
         <v>101</v>
       </c>
-      <c r="C14" s="61"/>
-      <c r="D14" s="61"/>
-      <c r="E14" s="61"/>
-      <c r="F14" s="61"/>
-      <c r="G14" s="61"/>
-      <c r="H14" s="61"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
     </row>
     <row r="15" spans="1:9" ht="19.5" customHeight="1">
       <c r="B15" s="21" t="s">
@@ -3808,13 +4076,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:D42"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -3823,19 +4091,19 @@
     <col min="5" max="6" width="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="22.9">
-      <c r="B2" s="64" t="s">
+    <row r="2" spans="2:4" ht="22.8">
+      <c r="B2" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
     </row>
     <row r="4" spans="2:4" ht="21.75" customHeight="1">
-      <c r="B4" s="66" t="s">
+      <c r="B4" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
     </row>
     <row r="5" spans="2:4" ht="18" customHeight="1">
       <c r="B5" s="23" t="s">
@@ -3904,11 +4172,11 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="21.75" customHeight="1">
-      <c r="B12" s="66" t="s">
+      <c r="B12" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="C12" s="66"/>
-      <c r="D12" s="66"/>
+      <c r="C12" s="63"/>
+      <c r="D12" s="63"/>
     </row>
     <row r="13" spans="2:4" ht="18" customHeight="1">
       <c r="B13" s="23" t="s">
@@ -3977,11 +4245,11 @@
       </c>
     </row>
     <row r="20" spans="2:4" ht="21.75" customHeight="1">
-      <c r="B20" s="66" t="s">
+      <c r="B20" s="63" t="s">
         <v>133</v>
       </c>
-      <c r="C20" s="66"/>
-      <c r="D20" s="66"/>
+      <c r="C20" s="63"/>
+      <c r="D20" s="63"/>
     </row>
     <row r="21" spans="2:4" ht="18" customHeight="1">
       <c r="B21" s="23" t="s">
@@ -4028,63 +4296,63 @@
       </c>
     </row>
     <row r="26" spans="2:4" ht="21.75" customHeight="1">
-      <c r="B26" s="66" t="s">
+      <c r="B26" s="63" t="s">
         <v>141</v>
       </c>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
+      <c r="C26" s="63"/>
+      <c r="D26" s="63"/>
     </row>
     <row r="27" spans="2:4" ht="18" customHeight="1">
-      <c r="B27" s="51" t="s">
+      <c r="B27" s="65" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="51"/>
+      <c r="C27" s="65"/>
       <c r="D27" s="23" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="28" spans="2:4" ht="30" customHeight="1">
-      <c r="B28" s="52" t="s">
+      <c r="B28" s="66" t="s">
         <v>55</v>
       </c>
-      <c r="C28" s="52"/>
+      <c r="C28" s="66"/>
       <c r="D28" s="25" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="30" customHeight="1">
-      <c r="B29" s="52" t="s">
+      <c r="B29" s="66" t="s">
         <v>73</v>
       </c>
-      <c r="C29" s="52"/>
+      <c r="C29" s="66"/>
       <c r="D29" s="25" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="30" customHeight="1">
-      <c r="B30" s="52" t="s">
+      <c r="B30" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="52"/>
+      <c r="C30" s="66"/>
       <c r="D30" s="25" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="30" customHeight="1">
-      <c r="B31" s="52" t="s">
+      <c r="B31" s="66" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="52"/>
+      <c r="C31" s="66"/>
       <c r="D31" s="25" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="21.75" customHeight="1">
-      <c r="B33" s="66" t="s">
+      <c r="B33" s="63" t="s">
         <v>147</v>
       </c>
-      <c r="C33" s="66"/>
-      <c r="D33" s="66"/>
+      <c r="C33" s="63"/>
+      <c r="D33" s="63"/>
     </row>
     <row r="34" spans="2:4" ht="18" customHeight="1">
       <c r="B34" s="23" t="s">
@@ -4164,19 +4432,14 @@
       </c>
     </row>
     <row r="42" spans="2:4" ht="27.75" customHeight="1">
-      <c r="B42" s="50" t="s">
+      <c r="B42" s="64" t="s">
         <v>167</v>
       </c>
-      <c r="C42" s="50"/>
-      <c r="D42" s="50"/>
+      <c r="C42" s="64"/>
+      <c r="D42" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B26:D26"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="B27:C27"/>
@@ -4184,6 +4447,11 @@
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B26:D26"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -4191,26 +4459,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c1ca8347-932d-4cf2-8518-970d0c875838">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="81b96442-d259-4d2f-847e-1d5aed50e7c0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100AD8ED9C7C9BE364D8BB8F77187059BFA" ma:contentTypeVersion="11" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a6f38d4d26a9334e060bee1eb5cd3c29">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c1ca8347-932d-4cf2-8518-970d0c875838" xmlns:ns3="81b96442-d259-4d2f-847e-1d5aed50e7c0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="210b7b7040cc406e9035bc144aaec4e5" ns2:_="" ns3:_="">
     <xsd:import namespace="c1ca8347-932d-4cf2-8518-970d0c875838"/>
@@ -4405,14 +4653,66 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c1ca8347-932d-4cf2-8518-970d0c875838">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="81b96442-d259-4d2f-847e-1d5aed50e7c0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15C7823E-6B84-49DF-87AD-AC5F1EEB0AA3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC6E54F1-8766-42CB-AAB3-BB0488F99479}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c1ca8347-932d-4cf2-8518-970d0c875838"/>
+    <ds:schemaRef ds:uri="81b96442-d259-4d2f-847e-1d5aed50e7c0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91C27A6E-367A-4315-B52F-1B3E74B2EDC7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91C27A6E-367A-4315-B52F-1B3E74B2EDC7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="81b96442-d259-4d2f-847e-1d5aed50e7c0"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="c1ca8347-932d-4cf2-8518-970d0c875838"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC6E54F1-8766-42CB-AAB3-BB0488F99479}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15C7823E-6B84-49DF-87AD-AC5F1EEB0AA3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>